<commit_message>
Update csf2627-timeline-template.xlsx with new data
</commit_message>
<xml_diff>
--- a/Timeline/csf2627-timeline-template.xlsx
+++ b/Timeline/csf2627-timeline-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josearaujo/Desktop/IST/MEIC/CSF/SharedFolderKali/CSF/Timeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6844BE64-3BD4-3042-87AF-2A0B657BC853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F00525E2-90CB-CB4E-B153-5A70EC521388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="1071">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="1072">
   <si>
     <t>Digital Forensics Timeline Lab1</t>
   </si>
@@ -3233,6 +3233,9 @@
   </si>
   <si>
     <t>ESP32_ADXL345_3Axis_Telemetry.xlsx (epstein_secret.py carrier) was created</t>
+  </si>
+  <si>
+    <t>Amelia's pdf was extracted with "pdfinfo amelia.pdf"</t>
   </si>
 </sst>
 </file>
@@ -3488,7 +3491,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3504,17 +3507,13 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -3522,19 +3521,19 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3559,13 +3558,21 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Lab1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="totalRow" dxfId="0"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="totalRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -3800,18 +3807,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="9"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="18"/>
     </row>
     <row r="2" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -3829,13 +3836,13 @@
       <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="17"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
@@ -3843,19 +3850,21 @@
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="12"/>
+        <v>13</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>1071</v>
+      </c>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="9"/>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
@@ -3863,19 +3872,19 @@
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="13"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="14"/>
+        <v>9</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="19"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="12"/>
     </row>
     <row r="5" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
@@ -3891,11 +3900,11 @@
       <c r="E5" s="6" t="s">
         <v>1067</v>
       </c>
-      <c r="F5" s="13"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="14"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
@@ -3911,11 +3920,11 @@
       <c r="E6" s="6" t="s">
         <v>1066</v>
       </c>
-      <c r="F6" s="13"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="14"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="12"/>
     </row>
     <row r="7" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
@@ -3931,11 +3940,11 @@
       <c r="E7" s="6" t="s">
         <v>1066</v>
       </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="14"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="12"/>
     </row>
     <row r="8" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
@@ -3951,11 +3960,11 @@
       <c r="E8" s="5" t="s">
         <v>1066</v>
       </c>
-      <c r="F8" s="13"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="14"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="12"/>
     </row>
     <row r="9" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
@@ -3971,11 +3980,11 @@
       <c r="E9" s="6" t="s">
         <v>1066</v>
       </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="14"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="12"/>
     </row>
     <row r="10" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
@@ -3991,11 +4000,11 @@
       <c r="E10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F10" s="13"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="14"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="12"/>
     </row>
     <row r="11" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
@@ -4011,11 +4020,11 @@
       <c r="E11" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="14"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="12"/>
     </row>
     <row r="12" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
@@ -4031,11 +4040,11 @@
       <c r="E12" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="13"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="14"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="12"/>
     </row>
     <row r="13" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
@@ -4051,11 +4060,11 @@
       <c r="E13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="13"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="14"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="12"/>
     </row>
     <row r="14" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
@@ -4071,11 +4080,11 @@
       <c r="E14" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F14" s="13"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="14"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="12"/>
     </row>
     <row r="15" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
@@ -4091,11 +4100,11 @@
       <c r="E15" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="14"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
@@ -4111,11 +4120,11 @@
       <c r="E16" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F16" s="13"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="14"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="12"/>
     </row>
     <row r="17" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
@@ -4131,11 +4140,11 @@
       <c r="E17" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="13"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="14"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
@@ -4151,11 +4160,11 @@
       <c r="E18" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F18" s="13"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="14"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="12"/>
     </row>
     <row r="19" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
@@ -4171,11 +4180,11 @@
       <c r="E19" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F19" s="13"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="14"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="12"/>
     </row>
     <row r="20" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
@@ -4191,11 +4200,11 @@
       <c r="E20" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="F20" s="15"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="17"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="15"/>
     </row>
     <row r="21" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
@@ -4211,11 +4220,11 @@
       <c r="E21" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F21" s="10"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="12"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="9"/>
     </row>
     <row r="22" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
@@ -4231,11 +4240,11 @@
       <c r="E22" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F22" s="13"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="14"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
@@ -4251,11 +4260,11 @@
       <c r="E23" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F23" s="13"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="14"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="12"/>
     </row>
     <row r="24" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
@@ -4271,11 +4280,11 @@
       <c r="E24" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="F24" s="13"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="14"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="12"/>
     </row>
     <row r="25" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
@@ -4291,11 +4300,11 @@
       <c r="E25" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F25" s="13"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="14"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="12"/>
     </row>
     <row r="26" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
@@ -4305,11 +4314,11 @@
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="14"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="12"/>
     </row>
     <row r="27" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
@@ -4319,11 +4328,11 @@
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="14"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="12"/>
     </row>
     <row r="28" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
@@ -4333,11 +4342,11 @@
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="14"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
@@ -4347,11 +4356,11 @@
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="14"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="12"/>
     </row>
     <row r="30" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
@@ -4361,11 +4370,11 @@
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="14"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
@@ -4375,11 +4384,11 @@
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
       <c r="E31" s="5"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
-      <c r="J31" s="14"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
+      <c r="J31" s="12"/>
     </row>
     <row r="32" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
@@ -4389,11 +4398,11 @@
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="14"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+      <c r="J32" s="12"/>
     </row>
     <row r="33" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
@@ -4403,11 +4412,11 @@
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
       <c r="E33" s="5"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="14"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+      <c r="J33" s="12"/>
     </row>
     <row r="34" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
@@ -4417,11 +4426,11 @@
       <c r="C34" s="5"/>
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="14"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="12"/>
     </row>
     <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
@@ -4431,11 +4440,11 @@
       <c r="C35" s="5"/>
       <c r="D35" s="5"/>
       <c r="E35" s="5"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="14"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
+      <c r="J35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
@@ -4445,11 +4454,11 @@
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
       <c r="E36" s="5"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="14"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+      <c r="J36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
@@ -4459,11 +4468,11 @@
       <c r="C37" s="5"/>
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="14"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+      <c r="J37" s="12"/>
     </row>
     <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
@@ -4473,11 +4482,11 @@
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="16"/>
-      <c r="H38" s="16"/>
-      <c r="I38" s="16"/>
-      <c r="J38" s="17"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="14"/>
+      <c r="J38" s="15"/>
     </row>
     <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
@@ -4487,11 +4496,11 @@
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-      <c r="J39" s="12"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="9"/>
     </row>
     <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
@@ -4501,11 +4510,11 @@
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="14"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+      <c r="J40" s="12"/>
     </row>
     <row r="41" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
@@ -4515,11 +4524,11 @@
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
-      <c r="I41" s="8"/>
-      <c r="J41" s="14"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
+      <c r="I41" s="11"/>
+      <c r="J41" s="12"/>
     </row>
     <row r="42" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
@@ -4529,11 +4538,11 @@
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="8"/>
-      <c r="I42" s="8"/>
-      <c r="J42" s="14"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
+      <c r="I42" s="11"/>
+      <c r="J42" s="12"/>
     </row>
     <row r="43" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
@@ -4543,11 +4552,11 @@
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="5"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="8"/>
-      <c r="I43" s="8"/>
-      <c r="J43" s="14"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="11"/>
+      <c r="H43" s="11"/>
+      <c r="I43" s="11"/>
+      <c r="J43" s="12"/>
     </row>
     <row r="44" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
@@ -4557,11 +4566,11 @@
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
       <c r="E44" s="5"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="8"/>
-      <c r="I44" s="8"/>
-      <c r="J44" s="14"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="11"/>
+      <c r="H44" s="11"/>
+      <c r="I44" s="11"/>
+      <c r="J44" s="12"/>
     </row>
     <row r="45" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
@@ -4571,11 +4580,11 @@
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="8"/>
-      <c r="I45" s="8"/>
-      <c r="J45" s="14"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="11"/>
+      <c r="H45" s="11"/>
+      <c r="I45" s="11"/>
+      <c r="J45" s="12"/>
     </row>
     <row r="46" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
@@ -4585,11 +4594,11 @@
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
       <c r="E46" s="5"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="8"/>
-      <c r="I46" s="8"/>
-      <c r="J46" s="14"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="11"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="11"/>
+      <c r="J46" s="12"/>
     </row>
     <row r="47" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
@@ -4599,11 +4608,11 @@
       <c r="C47" s="5"/>
       <c r="D47" s="5"/>
       <c r="E47" s="5"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="14"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="11"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
+      <c r="J47" s="12"/>
     </row>
     <row r="48" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
@@ -4613,11 +4622,11 @@
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
       <c r="E48" s="5"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="8"/>
-      <c r="H48" s="8"/>
-      <c r="I48" s="8"/>
-      <c r="J48" s="14"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="11"/>
+      <c r="H48" s="11"/>
+      <c r="I48" s="11"/>
+      <c r="J48" s="12"/>
     </row>
     <row r="49" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
@@ -4627,11 +4636,11 @@
       <c r="C49" s="5"/>
       <c r="D49" s="5"/>
       <c r="E49" s="5"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="8"/>
-      <c r="I49" s="8"/>
-      <c r="J49" s="14"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="11"/>
+      <c r="H49" s="11"/>
+      <c r="I49" s="11"/>
+      <c r="J49" s="12"/>
     </row>
     <row r="50" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
@@ -4641,11 +4650,11 @@
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
-      <c r="F50" s="13"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="8"/>
-      <c r="I50" s="8"/>
-      <c r="J50" s="14"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="11"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
+      <c r="J50" s="12"/>
     </row>
     <row r="51" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
@@ -4655,11 +4664,11 @@
       <c r="C51" s="5"/>
       <c r="D51" s="5"/>
       <c r="E51" s="5"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="8"/>
-      <c r="I51" s="8"/>
-      <c r="J51" s="14"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="12"/>
     </row>
     <row r="52" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
@@ -4669,11 +4678,11 @@
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="8"/>
-      <c r="H52" s="8"/>
-      <c r="I52" s="8"/>
-      <c r="J52" s="14"/>
+      <c r="F52" s="10"/>
+      <c r="G52" s="11"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
+      <c r="J52" s="12"/>
     </row>
     <row r="53" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
@@ -4683,11 +4692,11 @@
       <c r="C53" s="5"/>
       <c r="D53" s="5"/>
       <c r="E53" s="5"/>
-      <c r="F53" s="13"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="8"/>
-      <c r="I53" s="8"/>
-      <c r="J53" s="14"/>
+      <c r="F53" s="10"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="11"/>
+      <c r="J53" s="12"/>
     </row>
     <row r="54" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
@@ -4697,11 +4706,11 @@
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
       <c r="E54" s="5"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="8"/>
-      <c r="I54" s="8"/>
-      <c r="J54" s="14"/>
+      <c r="F54" s="10"/>
+      <c r="G54" s="11"/>
+      <c r="H54" s="11"/>
+      <c r="I54" s="11"/>
+      <c r="J54" s="12"/>
     </row>
     <row r="55" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
@@ -4711,11 +4720,11 @@
       <c r="C55" s="5"/>
       <c r="D55" s="5"/>
       <c r="E55" s="5"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="8"/>
-      <c r="H55" s="8"/>
-      <c r="I55" s="8"/>
-      <c r="J55" s="14"/>
+      <c r="F55" s="10"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="11"/>
+      <c r="I55" s="11"/>
+      <c r="J55" s="12"/>
     </row>
     <row r="56" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
@@ -4725,11 +4734,11 @@
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="16"/>
-      <c r="H56" s="16"/>
-      <c r="I56" s="16"/>
-      <c r="J56" s="17"/>
+      <c r="F56" s="13"/>
+      <c r="G56" s="14"/>
+      <c r="H56" s="14"/>
+      <c r="I56" s="14"/>
+      <c r="J56" s="15"/>
     </row>
     <row r="57" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
@@ -4739,11 +4748,11 @@
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
-      <c r="F57" s="10"/>
-      <c r="G57" s="11"/>
-      <c r="H57" s="11"/>
-      <c r="I57" s="11"/>
-      <c r="J57" s="12"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8"/>
+      <c r="I57" s="8"/>
+      <c r="J57" s="9"/>
     </row>
     <row r="58" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
@@ -4753,11 +4762,11 @@
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
       <c r="E58" s="5"/>
-      <c r="F58" s="13"/>
-      <c r="G58" s="8"/>
-      <c r="H58" s="8"/>
-      <c r="I58" s="8"/>
-      <c r="J58" s="14"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="12"/>
     </row>
     <row r="59" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
@@ -4767,11 +4776,11 @@
       <c r="C59" s="5"/>
       <c r="D59" s="5"/>
       <c r="E59" s="5"/>
-      <c r="F59" s="13"/>
-      <c r="G59" s="8"/>
-      <c r="H59" s="8"/>
-      <c r="I59" s="8"/>
-      <c r="J59" s="14"/>
+      <c r="F59" s="10"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="12"/>
     </row>
     <row r="60" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
@@ -4781,11 +4790,11 @@
       <c r="C60" s="5"/>
       <c r="D60" s="5"/>
       <c r="E60" s="5"/>
-      <c r="F60" s="13"/>
-      <c r="G60" s="8"/>
-      <c r="H60" s="8"/>
-      <c r="I60" s="8"/>
-      <c r="J60" s="14"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11"/>
+      <c r="I60" s="11"/>
+      <c r="J60" s="12"/>
     </row>
     <row r="61" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
@@ -4795,11 +4804,11 @@
       <c r="C61" s="5"/>
       <c r="D61" s="5"/>
       <c r="E61" s="5"/>
-      <c r="F61" s="13"/>
-      <c r="G61" s="8"/>
-      <c r="H61" s="8"/>
-      <c r="I61" s="8"/>
-      <c r="J61" s="14"/>
+      <c r="F61" s="10"/>
+      <c r="G61" s="11"/>
+      <c r="H61" s="11"/>
+      <c r="I61" s="11"/>
+      <c r="J61" s="12"/>
     </row>
     <row r="62" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
@@ -4809,11 +4818,11 @@
       <c r="C62" s="5"/>
       <c r="D62" s="5"/>
       <c r="E62" s="5"/>
-      <c r="F62" s="13"/>
-      <c r="G62" s="8"/>
-      <c r="H62" s="8"/>
-      <c r="I62" s="8"/>
-      <c r="J62" s="14"/>
+      <c r="F62" s="10"/>
+      <c r="G62" s="11"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="11"/>
+      <c r="J62" s="12"/>
     </row>
     <row r="63" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
@@ -4823,11 +4832,11 @@
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
       <c r="E63" s="5"/>
-      <c r="F63" s="13"/>
-      <c r="G63" s="8"/>
-      <c r="H63" s="8"/>
-      <c r="I63" s="8"/>
-      <c r="J63" s="14"/>
+      <c r="F63" s="10"/>
+      <c r="G63" s="11"/>
+      <c r="H63" s="11"/>
+      <c r="I63" s="11"/>
+      <c r="J63" s="12"/>
     </row>
     <row r="64" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
@@ -4837,11 +4846,11 @@
       <c r="C64" s="5"/>
       <c r="D64" s="5"/>
       <c r="E64" s="5"/>
-      <c r="F64" s="13"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
-      <c r="I64" s="8"/>
-      <c r="J64" s="14"/>
+      <c r="F64" s="10"/>
+      <c r="G64" s="11"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="11"/>
+      <c r="J64" s="12"/>
     </row>
     <row r="65" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
@@ -4851,11 +4860,11 @@
       <c r="C65" s="5"/>
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
-      <c r="F65" s="13"/>
-      <c r="G65" s="8"/>
-      <c r="H65" s="8"/>
-      <c r="I65" s="8"/>
-      <c r="J65" s="14"/>
+      <c r="F65" s="10"/>
+      <c r="G65" s="11"/>
+      <c r="H65" s="11"/>
+      <c r="I65" s="11"/>
+      <c r="J65" s="12"/>
     </row>
     <row r="66" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
@@ -4865,11 +4874,11 @@
       <c r="C66" s="5"/>
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
-      <c r="F66" s="13"/>
-      <c r="G66" s="8"/>
-      <c r="H66" s="8"/>
-      <c r="I66" s="8"/>
-      <c r="J66" s="14"/>
+      <c r="F66" s="10"/>
+      <c r="G66" s="11"/>
+      <c r="H66" s="11"/>
+      <c r="I66" s="11"/>
+      <c r="J66" s="12"/>
     </row>
     <row r="67" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
@@ -4879,11 +4888,11 @@
       <c r="C67" s="5"/>
       <c r="D67" s="5"/>
       <c r="E67" s="5"/>
-      <c r="F67" s="13"/>
-      <c r="G67" s="8"/>
-      <c r="H67" s="8"/>
-      <c r="I67" s="8"/>
-      <c r="J67" s="14"/>
+      <c r="F67" s="10"/>
+      <c r="G67" s="11"/>
+      <c r="H67" s="11"/>
+      <c r="I67" s="11"/>
+      <c r="J67" s="12"/>
     </row>
     <row r="68" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
@@ -4893,11 +4902,11 @@
       <c r="C68" s="5"/>
       <c r="D68" s="5"/>
       <c r="E68" s="5"/>
-      <c r="F68" s="13"/>
-      <c r="G68" s="8"/>
-      <c r="H68" s="8"/>
-      <c r="I68" s="8"/>
-      <c r="J68" s="14"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="11"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+      <c r="J68" s="12"/>
     </row>
     <row r="69" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
@@ -4907,11 +4916,11 @@
       <c r="C69" s="5"/>
       <c r="D69" s="5"/>
       <c r="E69" s="5"/>
-      <c r="F69" s="13"/>
-      <c r="G69" s="8"/>
-      <c r="H69" s="8"/>
-      <c r="I69" s="8"/>
-      <c r="J69" s="14"/>
+      <c r="F69" s="10"/>
+      <c r="G69" s="11"/>
+      <c r="H69" s="11"/>
+      <c r="I69" s="11"/>
+      <c r="J69" s="12"/>
     </row>
     <row r="70" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
@@ -4921,11 +4930,11 @@
       <c r="C70" s="5"/>
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
-      <c r="F70" s="13"/>
-      <c r="G70" s="8"/>
-      <c r="H70" s="8"/>
-      <c r="I70" s="8"/>
-      <c r="J70" s="14"/>
+      <c r="F70" s="10"/>
+      <c r="G70" s="11"/>
+      <c r="H70" s="11"/>
+      <c r="I70" s="11"/>
+      <c r="J70" s="12"/>
     </row>
     <row r="71" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
@@ -4935,11 +4944,11 @@
       <c r="C71" s="5"/>
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
-      <c r="F71" s="13"/>
-      <c r="G71" s="8"/>
-      <c r="H71" s="8"/>
-      <c r="I71" s="8"/>
-      <c r="J71" s="14"/>
+      <c r="F71" s="10"/>
+      <c r="G71" s="11"/>
+      <c r="H71" s="11"/>
+      <c r="I71" s="11"/>
+      <c r="J71" s="12"/>
     </row>
     <row r="72" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
@@ -4949,11 +4958,11 @@
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
-      <c r="F72" s="13"/>
-      <c r="G72" s="8"/>
-      <c r="H72" s="8"/>
-      <c r="I72" s="8"/>
-      <c r="J72" s="14"/>
+      <c r="F72" s="10"/>
+      <c r="G72" s="11"/>
+      <c r="H72" s="11"/>
+      <c r="I72" s="11"/>
+      <c r="J72" s="12"/>
     </row>
     <row r="73" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
@@ -4963,11 +4972,11 @@
       <c r="C73" s="5"/>
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
-      <c r="F73" s="13"/>
-      <c r="G73" s="8"/>
-      <c r="H73" s="8"/>
-      <c r="I73" s="8"/>
-      <c r="J73" s="14"/>
+      <c r="F73" s="10"/>
+      <c r="G73" s="11"/>
+      <c r="H73" s="11"/>
+      <c r="I73" s="11"/>
+      <c r="J73" s="12"/>
     </row>
     <row r="74" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
@@ -4977,11 +4986,11 @@
       <c r="C74" s="5"/>
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
-      <c r="F74" s="15"/>
-      <c r="G74" s="16"/>
-      <c r="H74" s="16"/>
-      <c r="I74" s="16"/>
-      <c r="J74" s="17"/>
+      <c r="F74" s="13"/>
+      <c r="G74" s="14"/>
+      <c r="H74" s="14"/>
+      <c r="I74" s="14"/>
+      <c r="J74" s="15"/>
     </row>
     <row r="75" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
@@ -4991,11 +5000,11 @@
       <c r="C75" s="5"/>
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
-      <c r="F75" s="10"/>
-      <c r="G75" s="11"/>
-      <c r="H75" s="11"/>
-      <c r="I75" s="11"/>
-      <c r="J75" s="12"/>
+      <c r="F75" s="7"/>
+      <c r="G75" s="8"/>
+      <c r="H75" s="8"/>
+      <c r="I75" s="8"/>
+      <c r="J75" s="9"/>
     </row>
     <row r="76" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
@@ -5005,11 +5014,11 @@
       <c r="C76" s="5"/>
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
-      <c r="F76" s="13"/>
-      <c r="G76" s="8"/>
-      <c r="H76" s="8"/>
-      <c r="I76" s="8"/>
-      <c r="J76" s="14"/>
+      <c r="F76" s="10"/>
+      <c r="G76" s="11"/>
+      <c r="H76" s="11"/>
+      <c r="I76" s="11"/>
+      <c r="J76" s="12"/>
     </row>
     <row r="77" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
@@ -5019,11 +5028,11 @@
       <c r="C77" s="5"/>
       <c r="D77" s="5"/>
       <c r="E77" s="5"/>
-      <c r="F77" s="13"/>
-      <c r="G77" s="8"/>
-      <c r="H77" s="8"/>
-      <c r="I77" s="8"/>
-      <c r="J77" s="14"/>
+      <c r="F77" s="10"/>
+      <c r="G77" s="11"/>
+      <c r="H77" s="11"/>
+      <c r="I77" s="11"/>
+      <c r="J77" s="12"/>
     </row>
     <row r="78" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
@@ -5033,11 +5042,11 @@
       <c r="C78" s="5"/>
       <c r="D78" s="5"/>
       <c r="E78" s="5"/>
-      <c r="F78" s="13"/>
-      <c r="G78" s="8"/>
-      <c r="H78" s="8"/>
-      <c r="I78" s="8"/>
-      <c r="J78" s="14"/>
+      <c r="F78" s="10"/>
+      <c r="G78" s="11"/>
+      <c r="H78" s="11"/>
+      <c r="I78" s="11"/>
+      <c r="J78" s="12"/>
     </row>
     <row r="79" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
@@ -5047,11 +5056,11 @@
       <c r="C79" s="5"/>
       <c r="D79" s="5"/>
       <c r="E79" s="5"/>
-      <c r="F79" s="13"/>
-      <c r="G79" s="8"/>
-      <c r="H79" s="8"/>
-      <c r="I79" s="8"/>
-      <c r="J79" s="14"/>
+      <c r="F79" s="10"/>
+      <c r="G79" s="11"/>
+      <c r="H79" s="11"/>
+      <c r="I79" s="11"/>
+      <c r="J79" s="12"/>
     </row>
     <row r="80" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
@@ -5061,11 +5070,11 @@
       <c r="C80" s="5"/>
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
-      <c r="F80" s="13"/>
-      <c r="G80" s="8"/>
-      <c r="H80" s="8"/>
-      <c r="I80" s="8"/>
-      <c r="J80" s="14"/>
+      <c r="F80" s="10"/>
+      <c r="G80" s="11"/>
+      <c r="H80" s="11"/>
+      <c r="I80" s="11"/>
+      <c r="J80" s="12"/>
     </row>
     <row r="81" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
@@ -5075,11 +5084,11 @@
       <c r="C81" s="5"/>
       <c r="D81" s="5"/>
       <c r="E81" s="5"/>
-      <c r="F81" s="13"/>
-      <c r="G81" s="8"/>
-      <c r="H81" s="8"/>
-      <c r="I81" s="8"/>
-      <c r="J81" s="14"/>
+      <c r="F81" s="10"/>
+      <c r="G81" s="11"/>
+      <c r="H81" s="11"/>
+      <c r="I81" s="11"/>
+      <c r="J81" s="12"/>
     </row>
     <row r="82" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
@@ -5089,11 +5098,11 @@
       <c r="C82" s="5"/>
       <c r="D82" s="5"/>
       <c r="E82" s="5"/>
-      <c r="F82" s="13"/>
-      <c r="G82" s="8"/>
-      <c r="H82" s="8"/>
-      <c r="I82" s="8"/>
-      <c r="J82" s="14"/>
+      <c r="F82" s="10"/>
+      <c r="G82" s="11"/>
+      <c r="H82" s="11"/>
+      <c r="I82" s="11"/>
+      <c r="J82" s="12"/>
     </row>
     <row r="83" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
@@ -5103,11 +5112,11 @@
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
       <c r="E83" s="5"/>
-      <c r="F83" s="13"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="8"/>
-      <c r="I83" s="8"/>
-      <c r="J83" s="14"/>
+      <c r="F83" s="10"/>
+      <c r="G83" s="11"/>
+      <c r="H83" s="11"/>
+      <c r="I83" s="11"/>
+      <c r="J83" s="12"/>
     </row>
     <row r="84" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
@@ -5117,11 +5126,11 @@
       <c r="C84" s="5"/>
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
-      <c r="F84" s="13"/>
-      <c r="G84" s="8"/>
-      <c r="H84" s="8"/>
-      <c r="I84" s="8"/>
-      <c r="J84" s="14"/>
+      <c r="F84" s="10"/>
+      <c r="G84" s="11"/>
+      <c r="H84" s="11"/>
+      <c r="I84" s="11"/>
+      <c r="J84" s="12"/>
     </row>
     <row r="85" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
@@ -5131,11 +5140,11 @@
       <c r="C85" s="5"/>
       <c r="D85" s="5"/>
       <c r="E85" s="5"/>
-      <c r="F85" s="13"/>
-      <c r="G85" s="8"/>
-      <c r="H85" s="8"/>
-      <c r="I85" s="8"/>
-      <c r="J85" s="14"/>
+      <c r="F85" s="10"/>
+      <c r="G85" s="11"/>
+      <c r="H85" s="11"/>
+      <c r="I85" s="11"/>
+      <c r="J85" s="12"/>
     </row>
     <row r="86" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
@@ -5145,11 +5154,11 @@
       <c r="C86" s="5"/>
       <c r="D86" s="5"/>
       <c r="E86" s="5"/>
-      <c r="F86" s="13"/>
-      <c r="G86" s="8"/>
-      <c r="H86" s="8"/>
-      <c r="I86" s="8"/>
-      <c r="J86" s="14"/>
+      <c r="F86" s="10"/>
+      <c r="G86" s="11"/>
+      <c r="H86" s="11"/>
+      <c r="I86" s="11"/>
+      <c r="J86" s="12"/>
     </row>
     <row r="87" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
@@ -5159,11 +5168,11 @@
       <c r="C87" s="5"/>
       <c r="D87" s="5"/>
       <c r="E87" s="5"/>
-      <c r="F87" s="13"/>
-      <c r="G87" s="8"/>
-      <c r="H87" s="8"/>
-      <c r="I87" s="8"/>
-      <c r="J87" s="14"/>
+      <c r="F87" s="10"/>
+      <c r="G87" s="11"/>
+      <c r="H87" s="11"/>
+      <c r="I87" s="11"/>
+      <c r="J87" s="12"/>
     </row>
     <row r="88" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
@@ -5173,11 +5182,11 @@
       <c r="C88" s="5"/>
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
-      <c r="F88" s="13"/>
-      <c r="G88" s="8"/>
-      <c r="H88" s="8"/>
-      <c r="I88" s="8"/>
-      <c r="J88" s="14"/>
+      <c r="F88" s="10"/>
+      <c r="G88" s="11"/>
+      <c r="H88" s="11"/>
+      <c r="I88" s="11"/>
+      <c r="J88" s="12"/>
     </row>
     <row r="89" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
@@ -5187,11 +5196,11 @@
       <c r="C89" s="5"/>
       <c r="D89" s="5"/>
       <c r="E89" s="5"/>
-      <c r="F89" s="13"/>
-      <c r="G89" s="8"/>
-      <c r="H89" s="8"/>
-      <c r="I89" s="8"/>
-      <c r="J89" s="14"/>
+      <c r="F89" s="10"/>
+      <c r="G89" s="11"/>
+      <c r="H89" s="11"/>
+      <c r="I89" s="11"/>
+      <c r="J89" s="12"/>
     </row>
     <row r="90" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
@@ -5201,11 +5210,11 @@
       <c r="C90" s="5"/>
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
-      <c r="F90" s="13"/>
-      <c r="G90" s="8"/>
-      <c r="H90" s="8"/>
-      <c r="I90" s="8"/>
-      <c r="J90" s="14"/>
+      <c r="F90" s="10"/>
+      <c r="G90" s="11"/>
+      <c r="H90" s="11"/>
+      <c r="I90" s="11"/>
+      <c r="J90" s="12"/>
     </row>
     <row r="91" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
@@ -5215,11 +5224,11 @@
       <c r="C91" s="5"/>
       <c r="D91" s="5"/>
       <c r="E91" s="5"/>
-      <c r="F91" s="13"/>
-      <c r="G91" s="8"/>
-      <c r="H91" s="8"/>
-      <c r="I91" s="8"/>
-      <c r="J91" s="14"/>
+      <c r="F91" s="10"/>
+      <c r="G91" s="11"/>
+      <c r="H91" s="11"/>
+      <c r="I91" s="11"/>
+      <c r="J91" s="12"/>
     </row>
     <row r="92" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
@@ -5229,11 +5238,11 @@
       <c r="C92" s="5"/>
       <c r="D92" s="5"/>
       <c r="E92" s="5"/>
-      <c r="F92" s="15"/>
-      <c r="G92" s="16"/>
-      <c r="H92" s="16"/>
-      <c r="I92" s="16"/>
-      <c r="J92" s="17"/>
+      <c r="F92" s="13"/>
+      <c r="G92" s="14"/>
+      <c r="H92" s="14"/>
+      <c r="I92" s="14"/>
+      <c r="J92" s="15"/>
     </row>
     <row r="93" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
@@ -5243,11 +5252,11 @@
       <c r="C93" s="5"/>
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
-      <c r="F93" s="10"/>
-      <c r="G93" s="11"/>
-      <c r="H93" s="11"/>
-      <c r="I93" s="11"/>
-      <c r="J93" s="12"/>
+      <c r="F93" s="7"/>
+      <c r="G93" s="8"/>
+      <c r="H93" s="8"/>
+      <c r="I93" s="8"/>
+      <c r="J93" s="9"/>
     </row>
     <row r="94" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
@@ -5257,11 +5266,11 @@
       <c r="C94" s="5"/>
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
-      <c r="F94" s="13"/>
-      <c r="G94" s="8"/>
-      <c r="H94" s="8"/>
-      <c r="I94" s="8"/>
-      <c r="J94" s="14"/>
+      <c r="F94" s="10"/>
+      <c r="G94" s="11"/>
+      <c r="H94" s="11"/>
+      <c r="I94" s="11"/>
+      <c r="J94" s="12"/>
     </row>
     <row r="95" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="4" t="s">
@@ -5271,11 +5280,11 @@
       <c r="C95" s="5"/>
       <c r="D95" s="5"/>
       <c r="E95" s="5"/>
-      <c r="F95" s="13"/>
-      <c r="G95" s="8"/>
-      <c r="H95" s="8"/>
-      <c r="I95" s="8"/>
-      <c r="J95" s="14"/>
+      <c r="F95" s="10"/>
+      <c r="G95" s="11"/>
+      <c r="H95" s="11"/>
+      <c r="I95" s="11"/>
+      <c r="J95" s="12"/>
     </row>
     <row r="96" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="4" t="s">
@@ -5285,11 +5294,11 @@
       <c r="C96" s="5"/>
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
-      <c r="F96" s="13"/>
-      <c r="G96" s="8"/>
-      <c r="H96" s="8"/>
-      <c r="I96" s="8"/>
-      <c r="J96" s="14"/>
+      <c r="F96" s="10"/>
+      <c r="G96" s="11"/>
+      <c r="H96" s="11"/>
+      <c r="I96" s="11"/>
+      <c r="J96" s="12"/>
     </row>
     <row r="97" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
@@ -5299,11 +5308,11 @@
       <c r="C97" s="5"/>
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
-      <c r="F97" s="13"/>
-      <c r="G97" s="8"/>
-      <c r="H97" s="8"/>
-      <c r="I97" s="8"/>
-      <c r="J97" s="14"/>
+      <c r="F97" s="10"/>
+      <c r="G97" s="11"/>
+      <c r="H97" s="11"/>
+      <c r="I97" s="11"/>
+      <c r="J97" s="12"/>
     </row>
     <row r="98" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
@@ -5313,11 +5322,11 @@
       <c r="C98" s="5"/>
       <c r="D98" s="5"/>
       <c r="E98" s="5"/>
-      <c r="F98" s="13"/>
-      <c r="G98" s="8"/>
-      <c r="H98" s="8"/>
-      <c r="I98" s="8"/>
-      <c r="J98" s="14"/>
+      <c r="F98" s="10"/>
+      <c r="G98" s="11"/>
+      <c r="H98" s="11"/>
+      <c r="I98" s="11"/>
+      <c r="J98" s="12"/>
     </row>
     <row r="99" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="4" t="s">
@@ -5327,11 +5336,11 @@
       <c r="C99" s="5"/>
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
-      <c r="F99" s="13"/>
-      <c r="G99" s="8"/>
-      <c r="H99" s="8"/>
-      <c r="I99" s="8"/>
-      <c r="J99" s="14"/>
+      <c r="F99" s="10"/>
+      <c r="G99" s="11"/>
+      <c r="H99" s="11"/>
+      <c r="I99" s="11"/>
+      <c r="J99" s="12"/>
     </row>
     <row r="100" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="4" t="s">
@@ -5341,11 +5350,11 @@
       <c r="C100" s="5"/>
       <c r="D100" s="5"/>
       <c r="E100" s="5"/>
-      <c r="F100" s="13"/>
-      <c r="G100" s="8"/>
-      <c r="H100" s="8"/>
-      <c r="I100" s="8"/>
-      <c r="J100" s="14"/>
+      <c r="F100" s="10"/>
+      <c r="G100" s="11"/>
+      <c r="H100" s="11"/>
+      <c r="I100" s="11"/>
+      <c r="J100" s="12"/>
     </row>
     <row r="101" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="4" t="s">
@@ -5355,11 +5364,11 @@
       <c r="C101" s="5"/>
       <c r="D101" s="5"/>
       <c r="E101" s="5"/>
-      <c r="F101" s="13"/>
-      <c r="G101" s="8"/>
-      <c r="H101" s="8"/>
-      <c r="I101" s="8"/>
-      <c r="J101" s="14"/>
+      <c r="F101" s="10"/>
+      <c r="G101" s="11"/>
+      <c r="H101" s="11"/>
+      <c r="I101" s="11"/>
+      <c r="J101" s="12"/>
     </row>
     <row r="102" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="4" t="s">
@@ -5369,11 +5378,11 @@
       <c r="C102" s="5"/>
       <c r="D102" s="5"/>
       <c r="E102" s="5"/>
-      <c r="F102" s="13"/>
-      <c r="G102" s="8"/>
-      <c r="H102" s="8"/>
-      <c r="I102" s="8"/>
-      <c r="J102" s="14"/>
+      <c r="F102" s="10"/>
+      <c r="G102" s="11"/>
+      <c r="H102" s="11"/>
+      <c r="I102" s="11"/>
+      <c r="J102" s="12"/>
     </row>
     <row r="103" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
@@ -5383,11 +5392,11 @@
       <c r="C103" s="5"/>
       <c r="D103" s="5"/>
       <c r="E103" s="5"/>
-      <c r="F103" s="13"/>
-      <c r="G103" s="8"/>
-      <c r="H103" s="8"/>
-      <c r="I103" s="8"/>
-      <c r="J103" s="14"/>
+      <c r="F103" s="10"/>
+      <c r="G103" s="11"/>
+      <c r="H103" s="11"/>
+      <c r="I103" s="11"/>
+      <c r="J103" s="12"/>
     </row>
     <row r="104" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
@@ -5397,11 +5406,11 @@
       <c r="C104" s="5"/>
       <c r="D104" s="5"/>
       <c r="E104" s="5"/>
-      <c r="F104" s="13"/>
-      <c r="G104" s="8"/>
-      <c r="H104" s="8"/>
-      <c r="I104" s="8"/>
-      <c r="J104" s="14"/>
+      <c r="F104" s="10"/>
+      <c r="G104" s="11"/>
+      <c r="H104" s="11"/>
+      <c r="I104" s="11"/>
+      <c r="J104" s="12"/>
     </row>
     <row r="105" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="4" t="s">
@@ -5411,11 +5420,11 @@
       <c r="C105" s="5"/>
       <c r="D105" s="5"/>
       <c r="E105" s="5"/>
-      <c r="F105" s="13"/>
-      <c r="G105" s="8"/>
-      <c r="H105" s="8"/>
-      <c r="I105" s="8"/>
-      <c r="J105" s="14"/>
+      <c r="F105" s="10"/>
+      <c r="G105" s="11"/>
+      <c r="H105" s="11"/>
+      <c r="I105" s="11"/>
+      <c r="J105" s="12"/>
     </row>
     <row r="106" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
@@ -5425,11 +5434,11 @@
       <c r="C106" s="5"/>
       <c r="D106" s="5"/>
       <c r="E106" s="5"/>
-      <c r="F106" s="13"/>
-      <c r="G106" s="8"/>
-      <c r="H106" s="8"/>
-      <c r="I106" s="8"/>
-      <c r="J106" s="14"/>
+      <c r="F106" s="10"/>
+      <c r="G106" s="11"/>
+      <c r="H106" s="11"/>
+      <c r="I106" s="11"/>
+      <c r="J106" s="12"/>
     </row>
     <row r="107" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
@@ -5439,11 +5448,11 @@
       <c r="C107" s="5"/>
       <c r="D107" s="5"/>
       <c r="E107" s="5"/>
-      <c r="F107" s="13"/>
-      <c r="G107" s="8"/>
-      <c r="H107" s="8"/>
-      <c r="I107" s="8"/>
-      <c r="J107" s="14"/>
+      <c r="F107" s="10"/>
+      <c r="G107" s="11"/>
+      <c r="H107" s="11"/>
+      <c r="I107" s="11"/>
+      <c r="J107" s="12"/>
     </row>
     <row r="108" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="4" t="s">
@@ -5453,11 +5462,11 @@
       <c r="C108" s="5"/>
       <c r="D108" s="5"/>
       <c r="E108" s="5"/>
-      <c r="F108" s="13"/>
-      <c r="G108" s="8"/>
-      <c r="H108" s="8"/>
-      <c r="I108" s="8"/>
-      <c r="J108" s="14"/>
+      <c r="F108" s="10"/>
+      <c r="G108" s="11"/>
+      <c r="H108" s="11"/>
+      <c r="I108" s="11"/>
+      <c r="J108" s="12"/>
     </row>
     <row r="109" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="4" t="s">
@@ -5467,11 +5476,11 @@
       <c r="C109" s="5"/>
       <c r="D109" s="5"/>
       <c r="E109" s="5"/>
-      <c r="F109" s="13"/>
-      <c r="G109" s="8"/>
-      <c r="H109" s="8"/>
-      <c r="I109" s="8"/>
-      <c r="J109" s="14"/>
+      <c r="F109" s="10"/>
+      <c r="G109" s="11"/>
+      <c r="H109" s="11"/>
+      <c r="I109" s="11"/>
+      <c r="J109" s="12"/>
     </row>
     <row r="110" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="4" t="s">
@@ -5481,11 +5490,11 @@
       <c r="C110" s="5"/>
       <c r="D110" s="5"/>
       <c r="E110" s="5"/>
-      <c r="F110" s="15"/>
-      <c r="G110" s="16"/>
-      <c r="H110" s="16"/>
-      <c r="I110" s="16"/>
-      <c r="J110" s="17"/>
+      <c r="F110" s="13"/>
+      <c r="G110" s="14"/>
+      <c r="H110" s="14"/>
+      <c r="I110" s="14"/>
+      <c r="J110" s="15"/>
     </row>
     <row r="111" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="4" t="s">
@@ -5495,11 +5504,11 @@
       <c r="C111" s="5"/>
       <c r="D111" s="5"/>
       <c r="E111" s="5"/>
-      <c r="F111" s="10"/>
-      <c r="G111" s="11"/>
-      <c r="H111" s="11"/>
-      <c r="I111" s="11"/>
-      <c r="J111" s="12"/>
+      <c r="F111" s="7"/>
+      <c r="G111" s="8"/>
+      <c r="H111" s="8"/>
+      <c r="I111" s="8"/>
+      <c r="J111" s="9"/>
     </row>
     <row r="112" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="4" t="s">
@@ -5509,11 +5518,11 @@
       <c r="C112" s="5"/>
       <c r="D112" s="5"/>
       <c r="E112" s="5"/>
-      <c r="F112" s="13"/>
-      <c r="G112" s="8"/>
-      <c r="H112" s="8"/>
-      <c r="I112" s="8"/>
-      <c r="J112" s="14"/>
+      <c r="F112" s="10"/>
+      <c r="G112" s="11"/>
+      <c r="H112" s="11"/>
+      <c r="I112" s="11"/>
+      <c r="J112" s="12"/>
     </row>
     <row r="113" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
@@ -5523,11 +5532,11 @@
       <c r="C113" s="5"/>
       <c r="D113" s="5"/>
       <c r="E113" s="5"/>
-      <c r="F113" s="13"/>
-      <c r="G113" s="8"/>
-      <c r="H113" s="8"/>
-      <c r="I113" s="8"/>
-      <c r="J113" s="14"/>
+      <c r="F113" s="10"/>
+      <c r="G113" s="11"/>
+      <c r="H113" s="11"/>
+      <c r="I113" s="11"/>
+      <c r="J113" s="12"/>
     </row>
     <row r="114" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="4" t="s">
@@ -5537,11 +5546,11 @@
       <c r="C114" s="5"/>
       <c r="D114" s="5"/>
       <c r="E114" s="5"/>
-      <c r="F114" s="13"/>
-      <c r="G114" s="8"/>
-      <c r="H114" s="8"/>
-      <c r="I114" s="8"/>
-      <c r="J114" s="14"/>
+      <c r="F114" s="10"/>
+      <c r="G114" s="11"/>
+      <c r="H114" s="11"/>
+      <c r="I114" s="11"/>
+      <c r="J114" s="12"/>
     </row>
     <row r="115" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
@@ -5551,11 +5560,11 @@
       <c r="C115" s="5"/>
       <c r="D115" s="5"/>
       <c r="E115" s="5"/>
-      <c r="F115" s="13"/>
-      <c r="G115" s="8"/>
-      <c r="H115" s="8"/>
-      <c r="I115" s="8"/>
-      <c r="J115" s="14"/>
+      <c r="F115" s="10"/>
+      <c r="G115" s="11"/>
+      <c r="H115" s="11"/>
+      <c r="I115" s="11"/>
+      <c r="J115" s="12"/>
     </row>
     <row r="116" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="4" t="s">
@@ -5565,11 +5574,11 @@
       <c r="C116" s="5"/>
       <c r="D116" s="5"/>
       <c r="E116" s="5"/>
-      <c r="F116" s="13"/>
-      <c r="G116" s="8"/>
-      <c r="H116" s="8"/>
-      <c r="I116" s="8"/>
-      <c r="J116" s="14"/>
+      <c r="F116" s="10"/>
+      <c r="G116" s="11"/>
+      <c r="H116" s="11"/>
+      <c r="I116" s="11"/>
+      <c r="J116" s="12"/>
     </row>
     <row r="117" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="4" t="s">
@@ -5579,11 +5588,11 @@
       <c r="C117" s="5"/>
       <c r="D117" s="5"/>
       <c r="E117" s="5"/>
-      <c r="F117" s="13"/>
-      <c r="G117" s="8"/>
-      <c r="H117" s="8"/>
-      <c r="I117" s="8"/>
-      <c r="J117" s="14"/>
+      <c r="F117" s="10"/>
+      <c r="G117" s="11"/>
+      <c r="H117" s="11"/>
+      <c r="I117" s="11"/>
+      <c r="J117" s="12"/>
     </row>
     <row r="118" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
@@ -5593,11 +5602,11 @@
       <c r="C118" s="5"/>
       <c r="D118" s="5"/>
       <c r="E118" s="5"/>
-      <c r="F118" s="13"/>
-      <c r="G118" s="8"/>
-      <c r="H118" s="8"/>
-      <c r="I118" s="8"/>
-      <c r="J118" s="14"/>
+      <c r="F118" s="10"/>
+      <c r="G118" s="11"/>
+      <c r="H118" s="11"/>
+      <c r="I118" s="11"/>
+      <c r="J118" s="12"/>
     </row>
     <row r="119" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="4" t="s">
@@ -5607,11 +5616,11 @@
       <c r="C119" s="5"/>
       <c r="D119" s="5"/>
       <c r="E119" s="5"/>
-      <c r="F119" s="13"/>
-      <c r="G119" s="8"/>
-      <c r="H119" s="8"/>
-      <c r="I119" s="8"/>
-      <c r="J119" s="14"/>
+      <c r="F119" s="10"/>
+      <c r="G119" s="11"/>
+      <c r="H119" s="11"/>
+      <c r="I119" s="11"/>
+      <c r="J119" s="12"/>
     </row>
     <row r="120" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="4" t="s">
@@ -5621,11 +5630,11 @@
       <c r="C120" s="5"/>
       <c r="D120" s="5"/>
       <c r="E120" s="5"/>
-      <c r="F120" s="13"/>
-      <c r="G120" s="8"/>
-      <c r="H120" s="8"/>
-      <c r="I120" s="8"/>
-      <c r="J120" s="14"/>
+      <c r="F120" s="10"/>
+      <c r="G120" s="11"/>
+      <c r="H120" s="11"/>
+      <c r="I120" s="11"/>
+      <c r="J120" s="12"/>
     </row>
     <row r="121" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="4" t="s">
@@ -5635,11 +5644,11 @@
       <c r="C121" s="5"/>
       <c r="D121" s="5"/>
       <c r="E121" s="5"/>
-      <c r="F121" s="13"/>
-      <c r="G121" s="8"/>
-      <c r="H121" s="8"/>
-      <c r="I121" s="8"/>
-      <c r="J121" s="14"/>
+      <c r="F121" s="10"/>
+      <c r="G121" s="11"/>
+      <c r="H121" s="11"/>
+      <c r="I121" s="11"/>
+      <c r="J121" s="12"/>
     </row>
     <row r="122" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="4" t="s">
@@ -5649,11 +5658,11 @@
       <c r="C122" s="5"/>
       <c r="D122" s="5"/>
       <c r="E122" s="5"/>
-      <c r="F122" s="13"/>
-      <c r="G122" s="8"/>
-      <c r="H122" s="8"/>
-      <c r="I122" s="8"/>
-      <c r="J122" s="14"/>
+      <c r="F122" s="10"/>
+      <c r="G122" s="11"/>
+      <c r="H122" s="11"/>
+      <c r="I122" s="11"/>
+      <c r="J122" s="12"/>
     </row>
     <row r="123" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="4" t="s">
@@ -5663,11 +5672,11 @@
       <c r="C123" s="5"/>
       <c r="D123" s="5"/>
       <c r="E123" s="5"/>
-      <c r="F123" s="13"/>
-      <c r="G123" s="8"/>
-      <c r="H123" s="8"/>
-      <c r="I123" s="8"/>
-      <c r="J123" s="14"/>
+      <c r="F123" s="10"/>
+      <c r="G123" s="11"/>
+      <c r="H123" s="11"/>
+      <c r="I123" s="11"/>
+      <c r="J123" s="12"/>
     </row>
     <row r="124" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="4" t="s">
@@ -5677,11 +5686,11 @@
       <c r="C124" s="5"/>
       <c r="D124" s="5"/>
       <c r="E124" s="5"/>
-      <c r="F124" s="13"/>
-      <c r="G124" s="8"/>
-      <c r="H124" s="8"/>
-      <c r="I124" s="8"/>
-      <c r="J124" s="14"/>
+      <c r="F124" s="10"/>
+      <c r="G124" s="11"/>
+      <c r="H124" s="11"/>
+      <c r="I124" s="11"/>
+      <c r="J124" s="12"/>
     </row>
     <row r="125" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
@@ -5691,11 +5700,11 @@
       <c r="C125" s="5"/>
       <c r="D125" s="5"/>
       <c r="E125" s="5"/>
-      <c r="F125" s="13"/>
-      <c r="G125" s="8"/>
-      <c r="H125" s="8"/>
-      <c r="I125" s="8"/>
-      <c r="J125" s="14"/>
+      <c r="F125" s="10"/>
+      <c r="G125" s="11"/>
+      <c r="H125" s="11"/>
+      <c r="I125" s="11"/>
+      <c r="J125" s="12"/>
     </row>
     <row r="126" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="4" t="s">
@@ -5705,11 +5714,11 @@
       <c r="C126" s="5"/>
       <c r="D126" s="5"/>
       <c r="E126" s="5"/>
-      <c r="F126" s="13"/>
-      <c r="G126" s="8"/>
-      <c r="H126" s="8"/>
-      <c r="I126" s="8"/>
-      <c r="J126" s="14"/>
+      <c r="F126" s="10"/>
+      <c r="G126" s="11"/>
+      <c r="H126" s="11"/>
+      <c r="I126" s="11"/>
+      <c r="J126" s="12"/>
     </row>
     <row r="127" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="4" t="s">
@@ -5719,11 +5728,11 @@
       <c r="C127" s="5"/>
       <c r="D127" s="5"/>
       <c r="E127" s="5"/>
-      <c r="F127" s="13"/>
-      <c r="G127" s="8"/>
-      <c r="H127" s="8"/>
-      <c r="I127" s="8"/>
-      <c r="J127" s="14"/>
+      <c r="F127" s="10"/>
+      <c r="G127" s="11"/>
+      <c r="H127" s="11"/>
+      <c r="I127" s="11"/>
+      <c r="J127" s="12"/>
     </row>
     <row r="128" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
@@ -5733,11 +5742,11 @@
       <c r="C128" s="5"/>
       <c r="D128" s="5"/>
       <c r="E128" s="5"/>
-      <c r="F128" s="15"/>
-      <c r="G128" s="16"/>
-      <c r="H128" s="16"/>
-      <c r="I128" s="16"/>
-      <c r="J128" s="17"/>
+      <c r="F128" s="13"/>
+      <c r="G128" s="14"/>
+      <c r="H128" s="14"/>
+      <c r="I128" s="14"/>
+      <c r="J128" s="15"/>
     </row>
     <row r="129" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="4" t="s">
@@ -5747,11 +5756,11 @@
       <c r="C129" s="5"/>
       <c r="D129" s="5"/>
       <c r="E129" s="5"/>
-      <c r="F129" s="10"/>
-      <c r="G129" s="11"/>
-      <c r="H129" s="11"/>
-      <c r="I129" s="11"/>
-      <c r="J129" s="12"/>
+      <c r="F129" s="7"/>
+      <c r="G129" s="8"/>
+      <c r="H129" s="8"/>
+      <c r="I129" s="8"/>
+      <c r="J129" s="9"/>
     </row>
     <row r="130" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="4" t="s">
@@ -5761,11 +5770,11 @@
       <c r="C130" s="5"/>
       <c r="D130" s="5"/>
       <c r="E130" s="5"/>
-      <c r="F130" s="13"/>
-      <c r="G130" s="8"/>
-      <c r="H130" s="8"/>
-      <c r="I130" s="8"/>
-      <c r="J130" s="14"/>
+      <c r="F130" s="10"/>
+      <c r="G130" s="11"/>
+      <c r="H130" s="11"/>
+      <c r="I130" s="11"/>
+      <c r="J130" s="12"/>
     </row>
     <row r="131" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="4" t="s">
@@ -5775,11 +5784,11 @@
       <c r="C131" s="5"/>
       <c r="D131" s="5"/>
       <c r="E131" s="5"/>
-      <c r="F131" s="13"/>
-      <c r="G131" s="8"/>
-      <c r="H131" s="8"/>
-      <c r="I131" s="8"/>
-      <c r="J131" s="14"/>
+      <c r="F131" s="10"/>
+      <c r="G131" s="11"/>
+      <c r="H131" s="11"/>
+      <c r="I131" s="11"/>
+      <c r="J131" s="12"/>
     </row>
     <row r="132" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="4" t="s">
@@ -5789,11 +5798,11 @@
       <c r="C132" s="5"/>
       <c r="D132" s="5"/>
       <c r="E132" s="5"/>
-      <c r="F132" s="13"/>
-      <c r="G132" s="8"/>
-      <c r="H132" s="8"/>
-      <c r="I132" s="8"/>
-      <c r="J132" s="14"/>
+      <c r="F132" s="10"/>
+      <c r="G132" s="11"/>
+      <c r="H132" s="11"/>
+      <c r="I132" s="11"/>
+      <c r="J132" s="12"/>
     </row>
     <row r="133" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="4" t="s">
@@ -5803,11 +5812,11 @@
       <c r="C133" s="5"/>
       <c r="D133" s="5"/>
       <c r="E133" s="5"/>
-      <c r="F133" s="13"/>
-      <c r="G133" s="8"/>
-      <c r="H133" s="8"/>
-      <c r="I133" s="8"/>
-      <c r="J133" s="14"/>
+      <c r="F133" s="10"/>
+      <c r="G133" s="11"/>
+      <c r="H133" s="11"/>
+      <c r="I133" s="11"/>
+      <c r="J133" s="12"/>
     </row>
     <row r="134" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="4" t="s">
@@ -5817,11 +5826,11 @@
       <c r="C134" s="5"/>
       <c r="D134" s="5"/>
       <c r="E134" s="5"/>
-      <c r="F134" s="13"/>
-      <c r="G134" s="8"/>
-      <c r="H134" s="8"/>
-      <c r="I134" s="8"/>
-      <c r="J134" s="14"/>
+      <c r="F134" s="10"/>
+      <c r="G134" s="11"/>
+      <c r="H134" s="11"/>
+      <c r="I134" s="11"/>
+      <c r="J134" s="12"/>
     </row>
     <row r="135" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="4" t="s">
@@ -5831,11 +5840,11 @@
       <c r="C135" s="5"/>
       <c r="D135" s="5"/>
       <c r="E135" s="5"/>
-      <c r="F135" s="13"/>
-      <c r="G135" s="8"/>
-      <c r="H135" s="8"/>
-      <c r="I135" s="8"/>
-      <c r="J135" s="14"/>
+      <c r="F135" s="10"/>
+      <c r="G135" s="11"/>
+      <c r="H135" s="11"/>
+      <c r="I135" s="11"/>
+      <c r="J135" s="12"/>
     </row>
     <row r="136" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
@@ -5845,11 +5854,11 @@
       <c r="C136" s="5"/>
       <c r="D136" s="5"/>
       <c r="E136" s="5"/>
-      <c r="F136" s="13"/>
-      <c r="G136" s="8"/>
-      <c r="H136" s="8"/>
-      <c r="I136" s="8"/>
-      <c r="J136" s="14"/>
+      <c r="F136" s="10"/>
+      <c r="G136" s="11"/>
+      <c r="H136" s="11"/>
+      <c r="I136" s="11"/>
+      <c r="J136" s="12"/>
     </row>
     <row r="137" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
@@ -5859,11 +5868,11 @@
       <c r="C137" s="5"/>
       <c r="D137" s="5"/>
       <c r="E137" s="5"/>
-      <c r="F137" s="13"/>
-      <c r="G137" s="8"/>
-      <c r="H137" s="8"/>
-      <c r="I137" s="8"/>
-      <c r="J137" s="14"/>
+      <c r="F137" s="10"/>
+      <c r="G137" s="11"/>
+      <c r="H137" s="11"/>
+      <c r="I137" s="11"/>
+      <c r="J137" s="12"/>
     </row>
     <row r="138" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="4" t="s">
@@ -5873,11 +5882,11 @@
       <c r="C138" s="5"/>
       <c r="D138" s="5"/>
       <c r="E138" s="5"/>
-      <c r="F138" s="13"/>
-      <c r="G138" s="8"/>
-      <c r="H138" s="8"/>
-      <c r="I138" s="8"/>
-      <c r="J138" s="14"/>
+      <c r="F138" s="10"/>
+      <c r="G138" s="11"/>
+      <c r="H138" s="11"/>
+      <c r="I138" s="11"/>
+      <c r="J138" s="12"/>
     </row>
     <row r="139" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
@@ -5887,11 +5896,11 @@
       <c r="C139" s="5"/>
       <c r="D139" s="5"/>
       <c r="E139" s="5"/>
-      <c r="F139" s="13"/>
-      <c r="G139" s="8"/>
-      <c r="H139" s="8"/>
-      <c r="I139" s="8"/>
-      <c r="J139" s="14"/>
+      <c r="F139" s="10"/>
+      <c r="G139" s="11"/>
+      <c r="H139" s="11"/>
+      <c r="I139" s="11"/>
+      <c r="J139" s="12"/>
     </row>
     <row r="140" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="4" t="s">
@@ -5901,11 +5910,11 @@
       <c r="C140" s="5"/>
       <c r="D140" s="5"/>
       <c r="E140" s="5"/>
-      <c r="F140" s="13"/>
-      <c r="G140" s="8"/>
-      <c r="H140" s="8"/>
-      <c r="I140" s="8"/>
-      <c r="J140" s="14"/>
+      <c r="F140" s="10"/>
+      <c r="G140" s="11"/>
+      <c r="H140" s="11"/>
+      <c r="I140" s="11"/>
+      <c r="J140" s="12"/>
     </row>
     <row r="141" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="4" t="s">
@@ -5915,11 +5924,11 @@
       <c r="C141" s="5"/>
       <c r="D141" s="5"/>
       <c r="E141" s="5"/>
-      <c r="F141" s="13"/>
-      <c r="G141" s="8"/>
-      <c r="H141" s="8"/>
-      <c r="I141" s="8"/>
-      <c r="J141" s="14"/>
+      <c r="F141" s="10"/>
+      <c r="G141" s="11"/>
+      <c r="H141" s="11"/>
+      <c r="I141" s="11"/>
+      <c r="J141" s="12"/>
     </row>
     <row r="142" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="4" t="s">
@@ -5929,11 +5938,11 @@
       <c r="C142" s="5"/>
       <c r="D142" s="5"/>
       <c r="E142" s="5"/>
-      <c r="F142" s="13"/>
-      <c r="G142" s="8"/>
-      <c r="H142" s="8"/>
-      <c r="I142" s="8"/>
-      <c r="J142" s="14"/>
+      <c r="F142" s="10"/>
+      <c r="G142" s="11"/>
+      <c r="H142" s="11"/>
+      <c r="I142" s="11"/>
+      <c r="J142" s="12"/>
     </row>
     <row r="143" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="4" t="s">
@@ -5943,11 +5952,11 @@
       <c r="C143" s="5"/>
       <c r="D143" s="5"/>
       <c r="E143" s="5"/>
-      <c r="F143" s="13"/>
-      <c r="G143" s="8"/>
-      <c r="H143" s="8"/>
-      <c r="I143" s="8"/>
-      <c r="J143" s="14"/>
+      <c r="F143" s="10"/>
+      <c r="G143" s="11"/>
+      <c r="H143" s="11"/>
+      <c r="I143" s="11"/>
+      <c r="J143" s="12"/>
     </row>
     <row r="144" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="4" t="s">
@@ -5957,11 +5966,11 @@
       <c r="C144" s="5"/>
       <c r="D144" s="5"/>
       <c r="E144" s="5"/>
-      <c r="F144" s="13"/>
-      <c r="G144" s="8"/>
-      <c r="H144" s="8"/>
-      <c r="I144" s="8"/>
-      <c r="J144" s="14"/>
+      <c r="F144" s="10"/>
+      <c r="G144" s="11"/>
+      <c r="H144" s="11"/>
+      <c r="I144" s="11"/>
+      <c r="J144" s="12"/>
     </row>
     <row r="145" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="4" t="s">
@@ -5971,11 +5980,11 @@
       <c r="C145" s="5"/>
       <c r="D145" s="5"/>
       <c r="E145" s="5"/>
-      <c r="F145" s="13"/>
-      <c r="G145" s="8"/>
-      <c r="H145" s="8"/>
-      <c r="I145" s="8"/>
-      <c r="J145" s="14"/>
+      <c r="F145" s="10"/>
+      <c r="G145" s="11"/>
+      <c r="H145" s="11"/>
+      <c r="I145" s="11"/>
+      <c r="J145" s="12"/>
     </row>
     <row r="146" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="4" t="s">
@@ -5985,11 +5994,11 @@
       <c r="C146" s="5"/>
       <c r="D146" s="5"/>
       <c r="E146" s="5"/>
-      <c r="F146" s="15"/>
-      <c r="G146" s="16"/>
-      <c r="H146" s="16"/>
-      <c r="I146" s="16"/>
-      <c r="J146" s="17"/>
+      <c r="F146" s="13"/>
+      <c r="G146" s="14"/>
+      <c r="H146" s="14"/>
+      <c r="I146" s="14"/>
+      <c r="J146" s="15"/>
     </row>
     <row r="147" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="4" t="s">
@@ -13679,16 +13688,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="F75:J92"/>
+    <mergeCell ref="F3:J20"/>
+    <mergeCell ref="F39:J56"/>
+    <mergeCell ref="F21:J38"/>
     <mergeCell ref="F111:J128"/>
     <mergeCell ref="F129:J146"/>
     <mergeCell ref="F57:J74"/>
     <mergeCell ref="F93:J110"/>
     <mergeCell ref="F2:J2"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="F75:J92"/>
-    <mergeCell ref="F3:J20"/>
-    <mergeCell ref="F39:J56"/>
-    <mergeCell ref="F21:J38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape"/>

</xml_diff>